<commit_message>
Release v1.2.0 — rename plugin id to paraqualis-gxp
- plugin.json / marketplace.json: plugin id paraqualis-skills -> paraqualis-gxp (broader GxP/CSV scope than Part 11)
- Install is now: /plugin install paraqualis-gxp@paraqualis (repo + 'paraqualis' marketplace unchanged)
- server_version() reads name+version from plugin.json (single source of truth)
- Updated install commands in README/OVERVIEW/PUBLISHING/CHANGELOG; bumped self-qualification pack to v1.2.0

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Qualification/docs/Qualification-Pack.xlsx
+++ b/Qualification/docs/Qualification-Pack.xlsx
@@ -729,7 +729,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>PASS: all fields, `version = 1.1.0`</t>
+          <t>PASS: all fields, `version = 1.2.0`</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Declared version (`1.1.0`) surfaced at runtime so deployed version is verifiable</t>
+          <t>Declared version (`1.2.0`) surfaced at runtime so deployed version is verifiable</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>PASS — `server_version()` → 1.1.0 / 3.12.13</t>
+          <t>PASS — `server_version()` → 1.2.0 / 3.12.13</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -4711,7 +4711,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>You cannot ask the running toolkit which version it is. The version (`1.1.0`) lives only in a static file; no running component reports it. In a regulated setting you must be able to confirm at any time that the version in use is the qualified one.</t>
+          <t>You cannot ask the running toolkit which version it is. The version (`1.2.0`) lives only in a static file; no running component reports it. In a regulated setting you must be able to confirm at any time that the version in use is the qualified one.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -4746,7 +4746,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Closed (2026-06-17) — `server_version()` MCP tool added; returns `plugin.json` version + Python runtime (verified 1.1.0 / 3.12.13).</t>
+          <t>Closed (2026-06-17) — `server_version()` MCP tool added; returns `plugin.json` version + Python runtime (verified 1.2.0 / 3.12.13).</t>
         </is>
       </c>
     </row>

</xml_diff>